<commit_message>
Added log(g) calculated using g=GM/R2 to ALLPARAMETERSfinal.csv
</commit_message>
<xml_diff>
--- a/tables/Important/ModelParameters.xlsx
+++ b/tables/Important/ModelParameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luukv\Documenten\NatuurSterrkenkundeMasterProject\CodeMP\MasterProject\tables\Important\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{26EF0ACA-4B96-4553-AF8A-A91B4870A689}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4F23474-7970-4D95-AAD1-148D214CDD01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="4275" windowWidth="21600" windowHeight="11325" xr2:uid="{2E9DE683-19D0-4887-88A1-E5DF71A9B3BA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{2E9DE683-19D0-4887-88A1-E5DF71A9B3BA}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>id</t>
   </si>
@@ -74,13 +74,16 @@
     <t>vsini</t>
   </si>
   <si>
-    <t>vsini_err</t>
-  </si>
-  <si>
     <t>V_rad</t>
   </si>
   <si>
     <t>V_rad_err</t>
+  </si>
+  <si>
+    <t>log(g)</t>
+  </si>
+  <si>
+    <t>vsini_logg</t>
   </si>
 </sst>
 </file>
@@ -452,7 +455,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EACEEA60-C874-41A5-B8DC-A25134879D89}">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -461,7 +464,7 @@
     <col min="5" max="5" width="18.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -478,19 +481,22 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" t="s">
         <v>11</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>12</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>13</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -506,14 +512,20 @@
       <c r="F2">
         <v>138</v>
       </c>
+      <c r="G2">
+        <v>148</v>
+      </c>
       <c r="H2">
         <v>166</v>
       </c>
       <c r="I2">
         <v>12</v>
       </c>
+      <c r="J2">
+        <v>2.8</v>
+      </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -529,14 +541,20 @@
       <c r="F3">
         <v>152</v>
       </c>
+      <c r="G3">
+        <v>152</v>
+      </c>
       <c r="H3">
         <v>-50</v>
       </c>
       <c r="I3">
         <v>24</v>
       </c>
+      <c r="J3">
+        <v>3.2</v>
+      </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -552,14 +570,20 @@
       <c r="F4">
         <v>208</v>
       </c>
+      <c r="G4">
+        <v>212</v>
+      </c>
       <c r="H4">
         <v>-1</v>
       </c>
       <c r="I4">
         <v>12</v>
       </c>
+      <c r="J4">
+        <v>3.2</v>
+      </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -575,14 +599,20 @@
       <c r="F5">
         <v>244</v>
       </c>
+      <c r="G5">
+        <v>216</v>
+      </c>
       <c r="H5">
         <v>315</v>
       </c>
       <c r="I5">
         <v>18</v>
       </c>
+      <c r="J5">
+        <v>3.2</v>
+      </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -598,14 +628,20 @@
       <c r="F6">
         <v>150</v>
       </c>
+      <c r="G6">
+        <v>150</v>
+      </c>
       <c r="H6">
         <v>188</v>
       </c>
       <c r="I6">
         <v>5</v>
       </c>
+      <c r="J6">
+        <v>3.2</v>
+      </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -621,11 +657,17 @@
       <c r="F7">
         <v>110</v>
       </c>
+      <c r="G7">
+        <v>110</v>
+      </c>
       <c r="H7">
         <v>-19</v>
       </c>
       <c r="I7">
         <v>6</v>
+      </c>
+      <c r="J7">
+        <v>3.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>